<commit_message>
Daily NSE scan: 2026-10-03
</commit_message>
<xml_diff>
--- a/output/2026-10-03/enriched_analysis.xlsx
+++ b/output/2026-10-03/enriched_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR50"/>
+  <dimension ref="A1:BR49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F2" t="n">
         <v>22</v>
@@ -889,25 +889,25 @@
         <v>86.05</v>
       </c>
       <c r="J2" t="n">
-        <v>76.3</v>
+        <v>77.33</v>
       </c>
       <c r="K2" t="n">
-        <v>12.8</v>
+        <v>11.3</v>
       </c>
       <c r="L2" t="n">
         <v>61.32</v>
       </c>
       <c r="M2" t="n">
-        <v>77.98999999999999</v>
+        <v>63.01</v>
       </c>
       <c r="N2" t="n">
-        <v>779924810</v>
+        <v>630053770</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>779924810</v>
+        <v>630053770</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -921,7 +921,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.728</v>
+        <v>2.204</v>
       </c>
       <c r="W2" t="n">
         <v>2859</v>
@@ -971,10 +971,10 @@
         <v>129.5</v>
       </c>
       <c r="AJ2" t="n">
-        <v>76.30180841958143</v>
+        <v>77.33020135925074</v>
       </c>
       <c r="AK2" t="n">
-        <v>12.8</v>
+        <v>11.3</v>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -1002,10 +1002,10 @@
         </is>
       </c>
       <c r="AQ2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AR2" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AS2" t="n">
         <v>24</v>
@@ -11485,16 +11485,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SANDUMA</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SANDUR MANGANESE &amp; IRON ORES LIMITED</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -11502,141 +11502,141 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="G48" t="n">
         <v>5</v>
       </c>
       <c r="H48" t="n">
-        <v>-13</v>
+        <v>-1</v>
       </c>
       <c r="I48" t="n">
-        <v>177.67</v>
+        <v>108.85</v>
       </c>
       <c r="J48" t="n">
-        <v>207.63</v>
+        <v>111.01</v>
       </c>
       <c r="K48" t="n">
-        <v>-14.4</v>
+        <v>-1.9</v>
       </c>
       <c r="L48" t="n">
-        <v>74.26000000000001</v>
+        <v>73.48</v>
       </c>
       <c r="M48" t="n">
-        <v>4.7</v>
+        <v>0.45</v>
       </c>
       <c r="N48" t="n">
-        <v>46970458</v>
+        <v>4484713</v>
       </c>
       <c r="O48" t="n">
-        <v>46898837</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>71621</v>
+        <v>4484713</v>
       </c>
       <c r="Q48" t="n">
-        <v>99.84999999999999</v>
+        <v>0</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Net Buying with Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S48" t="b">
         <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0</v>
+        <v>0.218</v>
       </c>
       <c r="W48" t="n">
-        <v>8637</v>
+        <v>206</v>
       </c>
       <c r="X48" t="n">
-        <v>14.6</v>
+        <v>24.6</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>
       </c>
       <c r="Z48" t="n">
-        <v>224</v>
+        <v>12.07</v>
       </c>
       <c r="AA48" t="n">
-        <v>38</v>
+        <v>-29</v>
       </c>
       <c r="AB48" t="n">
-        <v>3.32</v>
+        <v>1.02</v>
       </c>
       <c r="AC48" t="n">
-        <v>24.2</v>
+        <v>7.92</v>
       </c>
       <c r="AD48" t="n">
-        <v>0.11</v>
+        <v>0.98</v>
       </c>
       <c r="AE48" t="b">
         <v>1</v>
       </c>
       <c r="AF48" t="n">
-        <v>41</v>
+        <v>4.11</v>
       </c>
       <c r="AG48" t="n">
-        <v>197.42</v>
+        <v>112.05</v>
       </c>
       <c r="AH48" t="n">
-        <v>208.78</v>
+        <v>117.93</v>
       </c>
       <c r="AI48" t="n">
-        <v>3.4</v>
+        <v>6.5</v>
       </c>
       <c r="AJ48" t="n">
-        <v>207.6336012165256</v>
+        <v>111.0077475247525</v>
       </c>
       <c r="AK48" t="n">
-        <v>-14.4</v>
+        <v>-1.9</v>
       </c>
       <c r="AL48" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM48" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN48" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO48" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="AP48" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AQ48" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="AR48" t="n">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="AS48" t="n">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="AT48" t="n">
         <v>0</v>
@@ -11648,10 +11648,10 @@
         <v>0</v>
       </c>
       <c r="AW48" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AX48" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AY48" t="n">
         <v>0</v>
@@ -11663,10 +11663,10 @@
         <v>0</v>
       </c>
       <c r="BB48" t="n">
-        <v>0</v>
+        <v>4484713</v>
       </c>
       <c r="BC48" t="n">
-        <v>0</v>
+        <v>4484713</v>
       </c>
       <c r="BD48" t="n">
         <v>0</v>
@@ -11708,7 +11708,7 @@
         <v>1</v>
       </c>
       <c r="BQ48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BR48" t="n">
         <v>0</v>
@@ -11717,16 +11717,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>JINDAL STEEL LIMITED</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -11734,54 +11734,54 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="F49" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G49" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>-1</v>
+        <v>-18</v>
       </c>
       <c r="I49" t="n">
-        <v>108.85</v>
+        <v>1100.5</v>
       </c>
       <c r="J49" t="n">
-        <v>111.01</v>
+        <v>1157.18</v>
       </c>
       <c r="K49" t="n">
-        <v>-1.9</v>
+        <v>-4.9</v>
       </c>
       <c r="L49" t="n">
-        <v>73.48</v>
+        <v>61.21</v>
       </c>
       <c r="M49" t="n">
-        <v>0.45</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="N49" t="n">
-        <v>4484713</v>
+        <v>92111332</v>
       </c>
       <c r="O49" t="n">
-        <v>0</v>
+        <v>108203920</v>
       </c>
       <c r="P49" t="n">
-        <v>4484713</v>
+        <v>-16092588</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>117.47</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Net Buying</t>
+          <t>Net Selling</t>
         </is>
       </c>
       <c r="S49" t="b">
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -11789,52 +11789,52 @@
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0.218</v>
+        <v>0</v>
       </c>
       <c r="W49" t="n">
-        <v>206</v>
+        <v>112261</v>
       </c>
       <c r="X49" t="n">
-        <v>24.6</v>
+        <v>32.3</v>
       </c>
       <c r="Y49" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Z49" t="n">
-        <v>12.07</v>
+        <v>2224</v>
       </c>
       <c r="AA49" t="n">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="AB49" t="n">
-        <v>1.02</v>
+        <v>10.65</v>
       </c>
       <c r="AC49" t="n">
-        <v>7.92</v>
+        <v>10.8</v>
       </c>
       <c r="AD49" t="n">
-        <v>0.98</v>
+        <v>0.16</v>
       </c>
       <c r="AE49" t="b">
         <v>1</v>
       </c>
       <c r="AF49" t="n">
-        <v>4.11</v>
+        <v>15</v>
       </c>
       <c r="AG49" t="n">
-        <v>112.05</v>
+        <v>1123.81</v>
       </c>
       <c r="AH49" t="n">
-        <v>117.93</v>
+        <v>1135.91</v>
       </c>
       <c r="AI49" t="n">
-        <v>6.5</v>
+        <v>-1.1</v>
       </c>
       <c r="AJ49" t="n">
-        <v>111.0077475247525</v>
+        <v>1157.177537688442</v>
       </c>
       <c r="AK49" t="n">
-        <v>-1.9</v>
+        <v>-4.9</v>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
@@ -11843,17 +11843,17 @@
       </c>
       <c r="AM49" t="inlineStr">
         <is>
+          <t>Mature Accumulation</t>
+        </is>
+      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
           <t>Confirmed Accumulation</t>
         </is>
       </c>
-      <c r="AN49" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AP49" t="inlineStr">
@@ -11862,10 +11862,10 @@
         </is>
       </c>
       <c r="AQ49" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="AR49" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="AS49" t="n">
         <v>30</v>
@@ -11880,10 +11880,10 @@
         <v>0</v>
       </c>
       <c r="AW49" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AX49" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AY49" t="n">
         <v>0</v>
@@ -11895,10 +11895,10 @@
         <v>0</v>
       </c>
       <c r="BB49" t="n">
-        <v>4484713</v>
+        <v>92111332</v>
       </c>
       <c r="BC49" t="n">
-        <v>4484713</v>
+        <v>92111332</v>
       </c>
       <c r="BD49" t="n">
         <v>0</v>
@@ -11910,10 +11910,10 @@
         <v>0</v>
       </c>
       <c r="BG49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI49" t="n">
         <v>0</v>
@@ -11925,10 +11925,10 @@
         <v>0</v>
       </c>
       <c r="BL49" t="n">
-        <v>0</v>
+        <v>108203920</v>
       </c>
       <c r="BM49" t="n">
-        <v>0</v>
+        <v>108203920</v>
       </c>
       <c r="BN49" t="n">
         <v>0</v>
@@ -11940,241 +11940,9 @@
         <v>1</v>
       </c>
       <c r="BQ49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>JINDALSTEL</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>JINDAL STEEL LIMITED</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F50" t="n">
-        <v>12</v>
-      </c>
-      <c r="G50" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" t="n">
-        <v>-18</v>
-      </c>
-      <c r="I50" t="n">
-        <v>1100.5</v>
-      </c>
-      <c r="J50" t="n">
-        <v>1157.18</v>
-      </c>
-      <c r="K50" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="L50" t="n">
-        <v>61.21</v>
-      </c>
-      <c r="M50" t="n">
-        <v>9.210000000000001</v>
-      </c>
-      <c r="N50" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="O50" t="n">
-        <v>108203920</v>
-      </c>
-      <c r="P50" t="n">
-        <v>-16092588</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>117.47</v>
-      </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>Net Selling</t>
-        </is>
-      </c>
-      <c r="S50" t="b">
-        <v>0</v>
-      </c>
-      <c r="T50" t="n">
-        <v>1</v>
-      </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-      <c r="V50" t="n">
-        <v>0</v>
-      </c>
-      <c r="W50" t="n">
-        <v>112261</v>
-      </c>
-      <c r="X50" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="Y50" t="n">
-        <v>18</v>
-      </c>
-      <c r="Z50" t="n">
-        <v>2224</v>
-      </c>
-      <c r="AA50" t="n">
-        <v>-28</v>
-      </c>
-      <c r="AB50" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="AC50" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="AD50" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AE50" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF50" t="n">
-        <v>15</v>
-      </c>
-      <c r="AG50" t="n">
-        <v>1123.81</v>
-      </c>
-      <c r="AH50" t="n">
-        <v>1135.91</v>
-      </c>
-      <c r="AI50" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="AJ50" t="n">
-        <v>1157.177537688442</v>
-      </c>
-      <c r="AK50" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="AL50" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM50" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN50" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO50" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-      <c r="AP50" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR50" t="n">
-        <v>30</v>
-      </c>
-      <c r="AS50" t="n">
-        <v>30</v>
-      </c>
-      <c r="AT50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY50" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB50" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="BC50" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="BD50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BH50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL50" t="n">
-        <v>108203920</v>
-      </c>
-      <c r="BM50" t="n">
-        <v>108203920</v>
-      </c>
-      <c r="BN50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO50" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12189,7 +11957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12265,19 +12033,19 @@
         <v>86.05</v>
       </c>
       <c r="D2" t="n">
-        <v>76.3</v>
+        <v>77.33</v>
       </c>
       <c r="E2" t="n">
-        <v>12.8</v>
+        <v>11.3</v>
       </c>
       <c r="F2" t="n">
         <v>61.32</v>
       </c>
       <c r="G2" t="n">
-        <v>77.98999999999999</v>
+        <v>63.01</v>
       </c>
       <c r="H2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -13863,103 +13631,68 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SANDUMA</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SANDUR MANGANESE &amp; IRON ORES LIMITED</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>177.67</v>
+        <v>108.85</v>
       </c>
       <c r="D48" t="n">
-        <v>207.63</v>
+        <v>111.01</v>
       </c>
       <c r="E48" t="n">
-        <v>-14.4</v>
+        <v>-1.9</v>
       </c>
       <c r="F48" t="n">
-        <v>74.26000000000001</v>
+        <v>73.48</v>
       </c>
       <c r="G48" t="n">
-        <v>4.7</v>
+        <v>0.45</v>
       </c>
       <c r="H48" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>JINDAL STEEL LIMITED</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>108.85</v>
+        <v>1100.5</v>
       </c>
       <c r="D49" t="n">
-        <v>111.01</v>
+        <v>1157.18</v>
       </c>
       <c r="E49" t="n">
-        <v>-1.9</v>
+        <v>-4.9</v>
       </c>
       <c r="F49" t="n">
-        <v>73.48</v>
+        <v>61.21</v>
       </c>
       <c r="G49" t="n">
-        <v>0.45</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H49" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I49" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>JINDALSTEL</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>JINDAL STEEL LIMITED</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>1100.5</v>
-      </c>
-      <c r="D50" t="n">
-        <v>1157.18</v>
-      </c>
-      <c r="E50" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="F50" t="n">
-        <v>61.21</v>
-      </c>
-      <c r="G50" t="n">
-        <v>9.210000000000001</v>
-      </c>
-      <c r="H50" t="n">
-        <v>1</v>
-      </c>
-      <c r="I50" t="inlineStr">
         <is>
           <t>03-09-2026</t>
         </is>
@@ -14008,7 +13741,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -14038,7 +13771,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -14048,7 +13781,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">

</xml_diff>